<commit_message>
removed the $domain_lib_ccode variable from the output, adapted the test data and reran the tests successfully
</commit_message>
<xml_diff>
--- a/rules/CORE-000929/negative/01/data/unit-test-coreid-CG0001-negative.xlsx
+++ b/rules/CORE-000929/negative/01/data/unit-test-coreid-CG0001-negative.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/CORE-000929/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1233081D-47DF-A845-9962-2336BE24723E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD70ADCA-15C1-6E48-9C18-0B567F69FD9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1300" yWindow="660" windowWidth="28940" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="909" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="894" uniqueCount="253">
   <si>
     <t>Error group</t>
   </si>
@@ -56,12 +56,6 @@
   </si>
   <si>
     <t>C00004</t>
-  </si>
-  <si>
-    <t>$domain_lib_ccode</t>
-  </si>
-  <si>
-    <t>list of published DOMAIN CCODEs</t>
   </si>
   <si>
     <t>cm.xpt</t>
@@ -1292,26 +1286,26 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1326,26 +1320,26 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -1353,15 +1347,15 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1371,7 +1365,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -1399,7 +1393,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -1411,12 +1405,12 @@
         <v>8</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>12</v>
@@ -1428,18 +1422,18 @@
         <v>7</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
         <v>4</v>
@@ -1451,67 +1445,7 @@
         <v>8</v>
       </c>
       <c r="F4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" t="s">
         <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" t="s">
-        <v>4</v>
-      </c>
-      <c r="D7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1526,107 +1460,107 @@
   <sheetData>
     <row r="1" spans="1:11" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>31</v>
-      </c>
       <c r="D1" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="J1" s="16" t="s">
         <v>196</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="K1" s="16" t="s">
         <v>197</v>
-      </c>
-      <c r="J1" s="16" t="s">
-        <v>198</v>
-      </c>
-      <c r="K1" s="16" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="D2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>57</v>
-      </c>
       <c r="E2" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="G2" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="H2" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="I2" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="J2" s="17" t="s">
         <v>203</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="K2" s="17" t="s">
         <v>204</v>
-      </c>
-      <c r="J2" s="17" t="s">
-        <v>205</v>
-      </c>
-      <c r="K2" s="17" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="J3" s="17" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="K3" s="17" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
@@ -1666,29 +1600,29 @@
     </row>
     <row r="5" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="C5" s="15" t="s">
         <v>207</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>208</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>209</v>
       </c>
       <c r="D5" s="18">
         <v>1</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F5" s="21"/>
       <c r="G5" s="22">
         <v>100</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="J5" s="19">
         <v>37987</v>
@@ -1699,29 +1633,29 @@
     </row>
     <row r="6" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="C6" s="15" t="s">
         <v>207</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>208</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>209</v>
       </c>
       <c r="D6" s="18">
         <v>2</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F6" s="21"/>
       <c r="G6" s="22">
         <v>100</v>
       </c>
       <c r="H6" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="I6" s="15" t="s">
         <v>211</v>
-      </c>
-      <c r="I6" s="15" t="s">
-        <v>213</v>
       </c>
       <c r="J6" s="19">
         <v>37993</v>
@@ -1732,29 +1666,29 @@
     </row>
     <row r="7" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="C7" s="15" t="s">
         <v>207</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>208</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>209</v>
       </c>
       <c r="D7" s="18">
         <v>3</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F7" s="21"/>
       <c r="G7" s="22">
         <v>100</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="J7" s="19">
         <v>37995</v>
@@ -1765,29 +1699,29 @@
     </row>
     <row r="8" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D8" s="18">
         <v>1</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F8" s="21"/>
       <c r="G8" s="22">
         <v>100</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="J8" s="19">
         <v>37987</v>
@@ -1808,152 +1742,152 @@
   <sheetData>
     <row r="1" spans="1:16" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>31</v>
-      </c>
       <c r="D1" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="M1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="O1" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>224</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="96" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="D2" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>57</v>
-      </c>
       <c r="E2" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="G2" s="8" t="s">
         <v>227</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="H2" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="I2" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="J2" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="L2" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="M2" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="N2" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="O2" s="8" t="s">
         <v>231</v>
       </c>
-      <c r="J2" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="K2" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="L2" s="8" t="s">
+      <c r="P2" s="8" t="s">
         <v>232</v>
-      </c>
-      <c r="M2" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="N2" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="O2" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="P2" s="8" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="P3" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
@@ -2008,47 +1942,47 @@
     </row>
     <row r="5" spans="1:16" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>233</v>
+      </c>
+      <c r="C5" s="20" t="s">
         <v>81</v>
-      </c>
-      <c r="B5" s="20" t="s">
-        <v>235</v>
-      </c>
-      <c r="C5" s="20" t="s">
-        <v>83</v>
       </c>
       <c r="D5" s="20">
         <v>1</v>
       </c>
       <c r="E5" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="G5" s="20" t="s">
         <v>236</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="H5" s="20" t="s">
         <v>237</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="I5" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="H5" s="20" t="s">
+      <c r="J5" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="K5" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="L5" s="20" t="s">
         <v>239</v>
-      </c>
-      <c r="I5" s="20" t="s">
-        <v>240</v>
-      </c>
-      <c r="J5" s="20" t="s">
-        <v>94</v>
-      </c>
-      <c r="K5" s="20" t="s">
-        <v>94</v>
-      </c>
-      <c r="L5" s="20" t="s">
-        <v>241</v>
       </c>
       <c r="M5" s="15"/>
       <c r="N5" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O5" s="20" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="P5" s="20">
         <v>3</v>
@@ -2056,47 +1990,47 @@
     </row>
     <row r="6" spans="1:16" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>233</v>
+      </c>
+      <c r="C6" s="20" t="s">
         <v>81</v>
-      </c>
-      <c r="B6" s="20" t="s">
-        <v>235</v>
-      </c>
-      <c r="C6" s="20" t="s">
-        <v>83</v>
       </c>
       <c r="D6" s="20">
         <v>2</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="F6" s="20" t="s">
+        <v>241</v>
+      </c>
+      <c r="G6" s="20" t="s">
+        <v>242</v>
+      </c>
+      <c r="H6" s="20" t="s">
+        <v>237</v>
+      </c>
+      <c r="I6" s="20" t="s">
+        <v>238</v>
+      </c>
+      <c r="J6" s="20" t="s">
         <v>243</v>
       </c>
-      <c r="G6" s="20" t="s">
-        <v>244</v>
-      </c>
-      <c r="H6" s="20" t="s">
+      <c r="K6" s="20" t="s">
+        <v>243</v>
+      </c>
+      <c r="L6" s="20" t="s">
         <v>239</v>
-      </c>
-      <c r="I6" s="20" t="s">
-        <v>240</v>
-      </c>
-      <c r="J6" s="20" t="s">
-        <v>245</v>
-      </c>
-      <c r="K6" s="20" t="s">
-        <v>245</v>
-      </c>
-      <c r="L6" s="20" t="s">
-        <v>241</v>
       </c>
       <c r="M6" s="15"/>
       <c r="N6" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O6" s="20" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="P6" s="20">
         <v>3</v>
@@ -2104,47 +2038,47 @@
     </row>
     <row r="7" spans="1:16" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>233</v>
+      </c>
+      <c r="C7" s="20" t="s">
         <v>81</v>
-      </c>
-      <c r="B7" s="20" t="s">
-        <v>235</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>83</v>
       </c>
       <c r="D7" s="20">
         <v>3</v>
       </c>
       <c r="E7" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="G7" s="20" t="s">
         <v>236</v>
       </c>
-      <c r="F7" s="20" t="s">
-        <v>237</v>
-      </c>
-      <c r="G7" s="20" t="s">
+      <c r="H7" s="20" t="s">
+        <v>244</v>
+      </c>
+      <c r="I7" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="H7" s="20" t="s">
-        <v>246</v>
-      </c>
-      <c r="I7" s="20" t="s">
-        <v>240</v>
-      </c>
       <c r="J7" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="K7" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L7" s="20" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="M7" s="15"/>
       <c r="N7" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O7" s="20" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="P7" s="20">
         <v>3</v>
@@ -2152,47 +2086,47 @@
     </row>
     <row r="8" spans="1:16" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>233</v>
+      </c>
+      <c r="C8" s="20" t="s">
         <v>81</v>
-      </c>
-      <c r="B8" s="20" t="s">
-        <v>235</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>83</v>
       </c>
       <c r="D8" s="20">
         <v>4</v>
       </c>
       <c r="E8" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="F8" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="G8" s="20" t="s">
         <v>236</v>
       </c>
-      <c r="F8" s="20" t="s">
-        <v>237</v>
-      </c>
-      <c r="G8" s="20" t="s">
+      <c r="H8" s="20" t="s">
+        <v>246</v>
+      </c>
+      <c r="I8" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="H8" s="20" t="s">
-        <v>248</v>
-      </c>
-      <c r="I8" s="20" t="s">
-        <v>240</v>
-      </c>
       <c r="J8" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="K8" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L8" s="20" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="M8" s="15"/>
       <c r="N8" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O8" s="20" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="P8" s="20">
         <v>3</v>
@@ -2200,47 +2134,47 @@
     </row>
     <row r="9" spans="1:16" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>233</v>
+      </c>
+      <c r="C9" s="20" t="s">
         <v>81</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>235</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>83</v>
       </c>
       <c r="D9" s="20">
         <v>5</v>
       </c>
       <c r="E9" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="F9" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="G9" s="20" t="s">
         <v>236</v>
       </c>
-      <c r="F9" s="20" t="s">
-        <v>237</v>
-      </c>
-      <c r="G9" s="20" t="s">
+      <c r="H9" s="20" t="s">
+        <v>247</v>
+      </c>
+      <c r="I9" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="H9" s="20" t="s">
-        <v>249</v>
-      </c>
-      <c r="I9" s="20" t="s">
-        <v>240</v>
-      </c>
       <c r="J9" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="K9" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L9" s="20" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="M9" s="15"/>
       <c r="N9" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O9" s="20" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="P9" s="20">
         <v>3</v>
@@ -2248,47 +2182,47 @@
     </row>
     <row r="10" spans="1:16" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>233</v>
+      </c>
+      <c r="C10" s="20" t="s">
         <v>81</v>
-      </c>
-      <c r="B10" s="20" t="s">
-        <v>235</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>83</v>
       </c>
       <c r="D10" s="20">
         <v>6</v>
       </c>
       <c r="E10" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="G10" s="20" t="s">
         <v>236</v>
       </c>
-      <c r="F10" s="20" t="s">
-        <v>237</v>
-      </c>
-      <c r="G10" s="20" t="s">
+      <c r="H10" s="20" t="s">
+        <v>248</v>
+      </c>
+      <c r="I10" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="H10" s="20" t="s">
-        <v>250</v>
-      </c>
-      <c r="I10" s="20" t="s">
-        <v>240</v>
-      </c>
       <c r="J10" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="K10" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L10" s="20" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="M10" s="15"/>
       <c r="N10" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O10" s="20" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="P10" s="20">
         <v>3</v>
@@ -2296,47 +2230,47 @@
     </row>
     <row r="11" spans="1:16" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="20" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D11" s="20">
         <v>1</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="F11" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="G11" s="20" t="s">
+        <v>236</v>
+      </c>
+      <c r="H11" s="20" t="s">
         <v>237</v>
       </c>
-      <c r="G11" s="20" t="s">
+      <c r="I11" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="H11" s="20" t="s">
+      <c r="J11" s="20" t="s">
+        <v>245</v>
+      </c>
+      <c r="K11" s="20" t="s">
+        <v>245</v>
+      </c>
+      <c r="L11" s="20" t="s">
         <v>239</v>
-      </c>
-      <c r="I11" s="20" t="s">
-        <v>240</v>
-      </c>
-      <c r="J11" s="20" t="s">
-        <v>247</v>
-      </c>
-      <c r="K11" s="20" t="s">
-        <v>247</v>
-      </c>
-      <c r="L11" s="20" t="s">
-        <v>241</v>
       </c>
       <c r="M11" s="15"/>
       <c r="N11" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O11" s="20" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="P11" s="20">
         <v>2</v>
@@ -2344,47 +2278,47 @@
     </row>
     <row r="12" spans="1:16" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="20" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D12" s="20">
         <v>2</v>
       </c>
       <c r="E12" s="20" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="G12" s="20" t="s">
+        <v>236</v>
+      </c>
+      <c r="H12" s="20" t="s">
+        <v>244</v>
+      </c>
+      <c r="I12" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="H12" s="20" t="s">
-        <v>246</v>
-      </c>
-      <c r="I12" s="20" t="s">
-        <v>240</v>
-      </c>
       <c r="J12" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="K12" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L12" s="20" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="M12" s="15"/>
       <c r="N12" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O12" s="20" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="P12" s="20">
         <v>2</v>
@@ -2392,47 +2326,47 @@
     </row>
     <row r="13" spans="1:16" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="20" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D13" s="20">
         <v>3</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="G13" s="20" t="s">
+        <v>236</v>
+      </c>
+      <c r="H13" s="20" t="s">
+        <v>246</v>
+      </c>
+      <c r="I13" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="H13" s="20" t="s">
-        <v>248</v>
-      </c>
-      <c r="I13" s="20" t="s">
-        <v>240</v>
-      </c>
       <c r="J13" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="K13" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L13" s="20" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="M13" s="15"/>
       <c r="N13" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O13" s="20" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="P13" s="20">
         <v>2</v>
@@ -2440,47 +2374,47 @@
     </row>
     <row r="14" spans="1:16" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="20" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D14" s="20">
         <v>4</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="G14" s="20" t="s">
+        <v>236</v>
+      </c>
+      <c r="H14" s="20" t="s">
+        <v>247</v>
+      </c>
+      <c r="I14" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="H14" s="20" t="s">
-        <v>249</v>
-      </c>
-      <c r="I14" s="20" t="s">
-        <v>240</v>
-      </c>
       <c r="J14" s="20" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="K14" s="20" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L14" s="20" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="M14" s="15"/>
       <c r="N14" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O14" s="20" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="P14" s="20">
         <v>2</v>
@@ -2488,47 +2422,47 @@
     </row>
     <row r="15" spans="1:16" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="20" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D15" s="20">
         <v>5</v>
       </c>
       <c r="E15" s="20" t="s">
+        <v>250</v>
+      </c>
+      <c r="F15" s="20" t="s">
+        <v>241</v>
+      </c>
+      <c r="G15" s="20" t="s">
+        <v>242</v>
+      </c>
+      <c r="H15" s="20" t="s">
+        <v>247</v>
+      </c>
+      <c r="I15" s="20" t="s">
+        <v>238</v>
+      </c>
+      <c r="J15" s="20" t="s">
         <v>252</v>
       </c>
-      <c r="F15" s="20" t="s">
-        <v>243</v>
-      </c>
-      <c r="G15" s="20" t="s">
-        <v>244</v>
-      </c>
-      <c r="H15" s="20" t="s">
-        <v>249</v>
-      </c>
-      <c r="I15" s="20" t="s">
-        <v>240</v>
-      </c>
-      <c r="J15" s="20" t="s">
-        <v>254</v>
-      </c>
       <c r="K15" s="20" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="L15" s="20" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="M15" s="15"/>
       <c r="N15" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O15" s="20" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="P15" s="20">
         <v>2</v>
@@ -2536,47 +2470,47 @@
     </row>
     <row r="16" spans="1:16" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="20" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D16" s="20">
         <v>6</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="F16" s="20" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="G16" s="20" t="s">
+        <v>236</v>
+      </c>
+      <c r="H16" s="20" t="s">
+        <v>248</v>
+      </c>
+      <c r="I16" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="H16" s="20" t="s">
-        <v>250</v>
-      </c>
-      <c r="I16" s="20" t="s">
-        <v>240</v>
-      </c>
       <c r="J16" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="K16" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L16" s="20" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="M16" s="15"/>
       <c r="N16" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O16" s="20" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="P16" s="20">
         <v>2</v>
@@ -2594,197 +2528,197 @@
   <sheetData>
     <row r="1" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>31</v>
-      </c>
       <c r="D1" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="K1" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="L1" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="M1" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="T1" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="U1" s="4" t="s">
         <v>117</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="R1" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="96" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="D2" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>57</v>
-      </c>
       <c r="E2" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="G2" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="H2" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="I2" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="J2" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="K2" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="L2" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="M2" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="N2" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="O2" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="P2" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="M2" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="N2" s="8" t="s">
+      <c r="Q2" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="R2" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="S2" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="T2" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="O2" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="P2" s="8" t="s">
+      <c r="U2" s="8" t="s">
         <v>129</v>
-      </c>
-      <c r="Q2" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="R2" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="S2" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="T2" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="U2" s="8" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:21" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="P3" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="Q3" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="R3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="S3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="T3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="U3" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.2">
@@ -2854,31 +2788,31 @@
     </row>
     <row r="5" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D5" s="12">
         <v>1</v>
       </c>
       <c r="E5" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="G5" s="12" t="s">
         <v>133</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>135</v>
       </c>
       <c r="H5" s="12">
         <v>71</v>
       </c>
       <c r="I5" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J5" s="12">
         <v>71</v>
@@ -2887,7 +2821,7 @@
         <v>71</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M5" s="15"/>
       <c r="N5" s="15"/>
@@ -2897,13 +2831,13 @@
         <v>1</v>
       </c>
       <c r="R5" s="12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="S5" s="12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="T5" s="12" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="U5" s="12">
         <v>-7</v>
@@ -2911,31 +2845,31 @@
     </row>
     <row r="6" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D6" s="12">
         <v>2</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H6" s="12">
         <v>71</v>
       </c>
       <c r="I6" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J6" s="12">
         <v>71</v>
@@ -2944,7 +2878,7 @@
         <v>71</v>
       </c>
       <c r="L6" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M6" s="15"/>
       <c r="N6" s="15"/>
@@ -2954,13 +2888,13 @@
         <v>2</v>
       </c>
       <c r="R6" s="12" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="S6" s="12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="T6" s="12" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="U6" s="12">
         <v>-2</v>
@@ -2968,31 +2902,31 @@
     </row>
     <row r="7" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C7" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D7" s="12">
         <v>3</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H7" s="12">
         <v>83</v>
       </c>
       <c r="I7" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J7" s="12">
         <v>83</v>
@@ -3001,25 +2935,25 @@
         <v>83</v>
       </c>
       <c r="L7" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M7" s="15"/>
       <c r="N7" s="15"/>
       <c r="O7" s="12" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="P7" s="15"/>
       <c r="Q7" s="12">
         <v>3</v>
       </c>
       <c r="R7" s="12" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="S7" s="12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="T7" s="12" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="U7" s="12">
         <v>1</v>
@@ -3027,32 +2961,32 @@
     </row>
     <row r="8" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C8" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D8" s="12">
         <v>4</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F8" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="H8" s="12">
+        <v>79</v>
+      </c>
+      <c r="I8" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="G8" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="H8" s="12">
-        <v>79</v>
-      </c>
-      <c r="I8" s="12" t="s">
-        <v>136</v>
-      </c>
       <c r="J8" s="12">
         <v>79</v>
       </c>
@@ -3060,7 +2994,7 @@
         <v>79</v>
       </c>
       <c r="L8" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M8" s="15"/>
       <c r="N8" s="15"/>
@@ -3070,13 +3004,13 @@
         <v>4</v>
       </c>
       <c r="R8" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="S8" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="T8" s="12" t="s">
         <v>143</v>
-      </c>
-      <c r="S8" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="T8" s="12" t="s">
-        <v>145</v>
       </c>
       <c r="U8" s="12">
         <v>14</v>
@@ -3084,31 +3018,31 @@
     </row>
     <row r="9" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C9" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D9" s="12">
         <v>5</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H9" s="12">
         <v>68</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J9" s="12">
         <v>68</v>
@@ -3117,7 +3051,7 @@
         <v>68</v>
       </c>
       <c r="L9" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M9" s="15"/>
       <c r="N9" s="15"/>
@@ -3127,13 +3061,13 @@
         <v>5</v>
       </c>
       <c r="R9" s="12" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="S9" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T9" s="12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="U9" s="12">
         <v>27</v>
@@ -3141,32 +3075,32 @@
     </row>
     <row r="10" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C10" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D10" s="12">
         <v>6</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F10" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="H10" s="12">
+        <v>77</v>
+      </c>
+      <c r="I10" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="G10" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="H10" s="12">
-        <v>77</v>
-      </c>
-      <c r="I10" s="12" t="s">
-        <v>136</v>
-      </c>
       <c r="J10" s="12">
         <v>77</v>
       </c>
@@ -3174,7 +3108,7 @@
         <v>77</v>
       </c>
       <c r="L10" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M10" s="15"/>
       <c r="N10" s="15"/>
@@ -3186,13 +3120,13 @@
         <v>7</v>
       </c>
       <c r="R10" s="12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="S10" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T10" s="12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="U10" s="12">
         <v>42</v>
@@ -3200,31 +3134,31 @@
     </row>
     <row r="11" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C11" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D11" s="12">
         <v>7</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H11" s="12">
         <v>71</v>
       </c>
       <c r="I11" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J11" s="12">
         <v>71</v>
@@ -3233,7 +3167,7 @@
         <v>71</v>
       </c>
       <c r="L11" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M11" s="15"/>
       <c r="N11" s="15"/>
@@ -3245,13 +3179,13 @@
         <v>7</v>
       </c>
       <c r="R11" s="12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="S11" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T11" s="12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="U11" s="12">
         <v>42</v>
@@ -3259,31 +3193,31 @@
     </row>
     <row r="12" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C12" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D12" s="12">
         <v>8</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H12" s="12">
         <v>69</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J12" s="12">
         <v>69</v>
@@ -3292,7 +3226,7 @@
         <v>69</v>
       </c>
       <c r="L12" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M12" s="15"/>
       <c r="N12" s="15"/>
@@ -3304,13 +3238,13 @@
         <v>7</v>
       </c>
       <c r="R12" s="12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="S12" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T12" s="12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="U12" s="12">
         <v>42</v>
@@ -3318,31 +3252,31 @@
     </row>
     <row r="13" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C13" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D13" s="12">
         <v>9</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H13" s="12">
         <v>76</v>
       </c>
       <c r="I13" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J13" s="12">
         <v>76</v>
@@ -3351,7 +3285,7 @@
         <v>76</v>
       </c>
       <c r="L13" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M13" s="15"/>
       <c r="N13" s="15"/>
@@ -3363,13 +3297,13 @@
         <v>8</v>
       </c>
       <c r="R13" s="12" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="S13" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T13" s="12" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="U13" s="12">
         <v>55</v>
@@ -3377,31 +3311,31 @@
     </row>
     <row r="14" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C14" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D14" s="12">
         <v>20</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H14" s="12">
         <v>51</v>
       </c>
       <c r="I14" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J14" s="12">
         <v>51</v>
@@ -3410,7 +3344,7 @@
         <v>51</v>
       </c>
       <c r="L14" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="M14" s="15"/>
       <c r="N14" s="15"/>
@@ -3420,13 +3354,13 @@
         <v>5</v>
       </c>
       <c r="R14" s="12" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="S14" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T14" s="12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="U14" s="12">
         <v>27</v>
@@ -3434,31 +3368,31 @@
     </row>
     <row r="15" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C15" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D15" s="12">
         <v>21</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H15" s="12">
         <v>52</v>
       </c>
       <c r="I15" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J15" s="12">
         <v>52</v>
@@ -3467,7 +3401,7 @@
         <v>52</v>
       </c>
       <c r="L15" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="M15" s="15"/>
       <c r="N15" s="15"/>
@@ -3479,13 +3413,13 @@
         <v>7</v>
       </c>
       <c r="R15" s="12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="S15" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T15" s="12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="U15" s="12">
         <v>42</v>
@@ -3493,31 +3427,31 @@
     </row>
     <row r="16" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C16" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D16" s="12">
         <v>22</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H16" s="12">
         <v>62</v>
       </c>
       <c r="I16" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J16" s="12">
         <v>62</v>
@@ -3526,7 +3460,7 @@
         <v>62</v>
       </c>
       <c r="L16" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="M16" s="15"/>
       <c r="N16" s="15"/>
@@ -3538,13 +3472,13 @@
         <v>7</v>
       </c>
       <c r="R16" s="12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="S16" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T16" s="12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="U16" s="12">
         <v>42</v>
@@ -3552,31 +3486,31 @@
     </row>
     <row r="17" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C17" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D17" s="12">
         <v>23</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H17" s="12">
         <v>62</v>
       </c>
       <c r="I17" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J17" s="12">
         <v>62</v>
@@ -3585,7 +3519,7 @@
         <v>62</v>
       </c>
       <c r="L17" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="M17" s="15"/>
       <c r="N17" s="15"/>
@@ -3597,13 +3531,13 @@
         <v>7</v>
       </c>
       <c r="R17" s="12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="S17" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T17" s="12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="U17" s="12">
         <v>42</v>
@@ -3611,31 +3545,31 @@
     </row>
     <row r="18" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C18" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D18" s="12">
         <v>24</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H18" s="12">
         <v>50</v>
       </c>
       <c r="I18" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J18" s="12">
         <v>50</v>
@@ -3644,7 +3578,7 @@
         <v>50</v>
       </c>
       <c r="L18" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="M18" s="15"/>
       <c r="N18" s="15"/>
@@ -3656,13 +3590,13 @@
         <v>8</v>
       </c>
       <c r="R18" s="12" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="S18" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T18" s="12" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="U18" s="12">
         <v>55</v>
@@ -3670,31 +3604,31 @@
     </row>
     <row r="19" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C19" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D19" s="12">
         <v>25</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H19" s="12">
         <v>52</v>
       </c>
       <c r="I19" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J19" s="12">
         <v>52</v>
@@ -3703,7 +3637,7 @@
         <v>52</v>
       </c>
       <c r="L19" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="M19" s="15"/>
       <c r="N19" s="15"/>
@@ -3715,13 +3649,13 @@
         <v>8</v>
       </c>
       <c r="R19" s="12" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="S19" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T19" s="12" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="U19" s="12">
         <v>55</v>
@@ -3729,31 +3663,31 @@
     </row>
     <row r="20" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C20" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D20" s="12">
         <v>26</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H20" s="12">
         <v>54</v>
       </c>
       <c r="I20" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J20" s="12">
         <v>54</v>
@@ -3762,7 +3696,7 @@
         <v>54</v>
       </c>
       <c r="L20" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="M20" s="15"/>
       <c r="N20" s="15"/>
@@ -3774,13 +3708,13 @@
         <v>8</v>
       </c>
       <c r="R20" s="12" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="S20" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T20" s="12" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="U20" s="12">
         <v>55</v>
@@ -3788,32 +3722,32 @@
     </row>
     <row r="21" spans="1:21" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C21" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D21" s="12">
         <v>27</v>
       </c>
       <c r="E21" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="G21" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="H21" s="12">
+        <v>79</v>
+      </c>
+      <c r="I21" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="F21" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="G21" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="H21" s="12">
-        <v>79</v>
-      </c>
-      <c r="I21" s="12" t="s">
-        <v>156</v>
-      </c>
       <c r="J21" s="12">
         <v>79</v>
       </c>
@@ -3821,7 +3755,7 @@
         <v>79</v>
       </c>
       <c r="L21" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="M21" s="15"/>
       <c r="N21" s="15"/>
@@ -3833,13 +3767,13 @@
         <v>201</v>
       </c>
       <c r="R21" s="12" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="S21" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T21" s="12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="U21" s="12">
         <v>172</v>
@@ -3847,31 +3781,31 @@
     </row>
     <row r="22" spans="1:21" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C22" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D22" s="12">
         <v>28</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H22" s="12">
         <v>98</v>
       </c>
       <c r="I22" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J22" s="12">
         <v>98</v>
@@ -3880,7 +3814,7 @@
         <v>98</v>
       </c>
       <c r="L22" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="M22" s="15"/>
       <c r="N22" s="15"/>
@@ -3892,13 +3826,13 @@
         <v>201</v>
       </c>
       <c r="R22" s="12" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="S22" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T22" s="12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="U22" s="12">
         <v>172</v>
@@ -3906,31 +3840,31 @@
     </row>
     <row r="23" spans="1:21" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C23" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D23" s="12">
         <v>29</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H23" s="12">
         <v>94</v>
       </c>
       <c r="I23" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J23" s="12">
         <v>94</v>
@@ -3939,7 +3873,7 @@
         <v>94</v>
       </c>
       <c r="L23" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="M23" s="15"/>
       <c r="N23" s="15"/>
@@ -3951,13 +3885,13 @@
         <v>201</v>
       </c>
       <c r="R23" s="12" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="S23" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T23" s="12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="U23" s="12">
         <v>172</v>
@@ -3965,31 +3899,31 @@
     </row>
     <row r="24" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C24" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D24" s="12">
         <v>30</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H24" s="12">
         <v>137</v>
       </c>
       <c r="I24" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J24" s="12">
         <v>137</v>
@@ -3998,7 +3932,7 @@
         <v>137</v>
       </c>
       <c r="L24" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M24" s="15"/>
       <c r="N24" s="15"/>
@@ -4008,13 +3942,13 @@
         <v>1</v>
       </c>
       <c r="R24" s="12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="S24" s="12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="T24" s="12" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="U24" s="12">
         <v>-7</v>
@@ -4022,31 +3956,31 @@
     </row>
     <row r="25" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C25" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D25" s="12">
         <v>31</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H25" s="12">
         <v>137</v>
       </c>
       <c r="I25" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J25" s="12">
         <v>137</v>
@@ -4055,7 +3989,7 @@
         <v>137</v>
       </c>
       <c r="L25" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M25" s="15"/>
       <c r="N25" s="15"/>
@@ -4065,13 +3999,13 @@
         <v>2</v>
       </c>
       <c r="R25" s="12" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="S25" s="12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="T25" s="12" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="U25" s="12">
         <v>-2</v>
@@ -4079,31 +4013,31 @@
     </row>
     <row r="26" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C26" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D26" s="12">
         <v>32</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H26" s="12">
         <v>130</v>
       </c>
       <c r="I26" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J26" s="12">
         <v>130</v>
@@ -4112,25 +4046,25 @@
         <v>130</v>
       </c>
       <c r="L26" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M26" s="15"/>
       <c r="N26" s="15"/>
       <c r="O26" s="12" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="P26" s="15"/>
       <c r="Q26" s="12">
         <v>3</v>
       </c>
       <c r="R26" s="12" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="S26" s="12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="T26" s="12" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="U26" s="12">
         <v>1</v>
@@ -4138,58 +4072,58 @@
     </row>
     <row r="27" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C27" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B27" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D27" s="12">
         <v>46</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G27" s="15"/>
       <c r="H27" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="I27" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="J27" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="I27" s="12" t="s">
+      <c r="K27" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="J27" s="13" t="s">
+      <c r="L27" s="12" t="s">
         <v>166</v>
-      </c>
-      <c r="K27" s="13" t="s">
-        <v>167</v>
-      </c>
-      <c r="L27" s="12" t="s">
-        <v>168</v>
       </c>
       <c r="M27" s="15"/>
       <c r="N27" s="12" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="O27" s="12" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="P27" s="15"/>
       <c r="Q27" s="12">
         <v>3</v>
       </c>
       <c r="R27" s="12" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="S27" s="12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="T27" s="12" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="U27" s="12">
         <v>1</v>
@@ -4197,42 +4131,42 @@
     </row>
     <row r="28" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C28" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D28" s="12">
         <v>47</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G28" s="15"/>
       <c r="H28" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="I28" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="J28" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="I28" s="12" t="s">
+      <c r="K28" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="J28" s="13" t="s">
+      <c r="L28" s="12" t="s">
         <v>166</v>
-      </c>
-      <c r="K28" s="13" t="s">
-        <v>167</v>
-      </c>
-      <c r="L28" s="12" t="s">
-        <v>168</v>
       </c>
       <c r="M28" s="15"/>
       <c r="N28" s="12" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="O28" s="15"/>
       <c r="P28" s="15"/>
@@ -4240,13 +4174,13 @@
         <v>4</v>
       </c>
       <c r="R28" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="S28" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="T28" s="12" t="s">
         <v>143</v>
-      </c>
-      <c r="S28" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="T28" s="12" t="s">
-        <v>145</v>
       </c>
       <c r="U28" s="12">
         <v>14</v>
@@ -4254,42 +4188,42 @@
     </row>
     <row r="29" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C29" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D29" s="12">
         <v>48</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G29" s="15"/>
       <c r="H29" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="I29" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="J29" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="K29" s="13" t="s">
         <v>170</v>
       </c>
-      <c r="I29" s="12" t="s">
-        <v>165</v>
-      </c>
-      <c r="J29" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="K29" s="13" t="s">
-        <v>172</v>
-      </c>
       <c r="L29" s="12" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="M29" s="15"/>
       <c r="N29" s="12" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="O29" s="15"/>
       <c r="P29" s="15"/>
@@ -4297,13 +4231,13 @@
         <v>5</v>
       </c>
       <c r="R29" s="12" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="S29" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T29" s="12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="U29" s="12">
         <v>27</v>
@@ -4311,42 +4245,42 @@
     </row>
     <row r="30" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C30" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B30" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C30" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D30" s="12">
         <v>49</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G30" s="15"/>
       <c r="H30" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="I30" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="J30" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="K30" s="13" t="s">
         <v>173</v>
       </c>
-      <c r="I30" s="12" t="s">
-        <v>165</v>
-      </c>
-      <c r="J30" s="13" t="s">
-        <v>174</v>
-      </c>
-      <c r="K30" s="13" t="s">
-        <v>175</v>
-      </c>
       <c r="L30" s="12" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="M30" s="15"/>
       <c r="N30" s="12" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="O30" s="15"/>
       <c r="P30" s="15"/>
@@ -4354,13 +4288,13 @@
         <v>7</v>
       </c>
       <c r="R30" s="12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="S30" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T30" s="12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="U30" s="12">
         <v>42</v>
@@ -4368,42 +4302,42 @@
     </row>
     <row r="31" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C31" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B31" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C31" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D31" s="12">
         <v>50</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F31" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G31" s="15"/>
       <c r="H31" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="I31" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="J31" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="K31" s="13" t="s">
         <v>173</v>
       </c>
-      <c r="I31" s="12" t="s">
-        <v>165</v>
-      </c>
-      <c r="J31" s="13" t="s">
-        <v>174</v>
-      </c>
-      <c r="K31" s="13" t="s">
-        <v>175</v>
-      </c>
       <c r="L31" s="12" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="M31" s="15"/>
       <c r="N31" s="12" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="O31" s="15"/>
       <c r="P31" s="15"/>
@@ -4411,13 +4345,13 @@
         <v>8</v>
       </c>
       <c r="R31" s="12" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="S31" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T31" s="12" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="U31" s="12">
         <v>55</v>
@@ -4425,42 +4359,42 @@
     </row>
     <row r="32" spans="1:21" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C32" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C32" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D32" s="12">
         <v>51</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G32" s="15"/>
       <c r="H32" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="I32" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="J32" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="K32" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="I32" s="12" t="s">
-        <v>165</v>
-      </c>
-      <c r="J32" s="13" t="s">
-        <v>177</v>
-      </c>
-      <c r="K32" s="13" t="s">
-        <v>178</v>
-      </c>
       <c r="L32" s="12" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="M32" s="15"/>
       <c r="N32" s="12" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="O32" s="15"/>
       <c r="P32" s="15"/>
@@ -4468,13 +4402,13 @@
         <v>201</v>
       </c>
       <c r="R32" s="12" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="S32" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T32" s="12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="U32" s="12">
         <v>172</v>
@@ -4482,38 +4416,38 @@
     </row>
     <row r="33" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C33" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C33" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D33" s="12">
         <v>52</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G33" s="15"/>
       <c r="H33" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="I33" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="J33" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="I33" s="12" t="s">
+      <c r="K33" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="J33" s="13" t="s">
+      <c r="L33" s="12" t="s">
         <v>183</v>
-      </c>
-      <c r="K33" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="L33" s="12" t="s">
-        <v>185</v>
       </c>
       <c r="M33" s="15"/>
       <c r="N33" s="15"/>
@@ -4523,13 +4457,13 @@
         <v>1</v>
       </c>
       <c r="R33" s="12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="S33" s="12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="T33" s="12" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="U33" s="12">
         <v>-7</v>
@@ -4537,56 +4471,56 @@
     </row>
     <row r="34" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C34" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B34" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C34" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D34" s="12">
         <v>53</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G34" s="15"/>
       <c r="H34" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="I34" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="J34" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="K34" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="I34" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="J34" s="13" t="s">
-        <v>187</v>
-      </c>
-      <c r="K34" s="13" t="s">
-        <v>188</v>
-      </c>
       <c r="L34" s="12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="M34" s="15"/>
       <c r="N34" s="15"/>
       <c r="O34" s="12" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="P34" s="15"/>
       <c r="Q34" s="12">
         <v>3</v>
       </c>
       <c r="R34" s="12" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="S34" s="12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="T34" s="12" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="U34" s="12">
         <v>1</v>
@@ -4594,38 +4528,38 @@
     </row>
     <row r="35" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C35" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D35" s="12">
         <v>54</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F35" s="12" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G35" s="15"/>
       <c r="H35" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="I35" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="J35" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="K35" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="I35" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="J35" s="13" t="s">
-        <v>187</v>
-      </c>
-      <c r="K35" s="13" t="s">
-        <v>188</v>
-      </c>
       <c r="L35" s="12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="M35" s="15"/>
       <c r="N35" s="15"/>
@@ -4635,13 +4569,13 @@
         <v>4</v>
       </c>
       <c r="R35" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="S35" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="T35" s="12" t="s">
         <v>143</v>
-      </c>
-      <c r="S35" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="T35" s="12" t="s">
-        <v>145</v>
       </c>
       <c r="U35" s="12">
         <v>14</v>
@@ -4649,38 +4583,38 @@
     </row>
     <row r="36" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C36" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C36" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D36" s="12">
         <v>55</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G36" s="15"/>
       <c r="H36" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="I36" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="J36" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="K36" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="I36" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="J36" s="13" t="s">
-        <v>190</v>
-      </c>
-      <c r="K36" s="13" t="s">
-        <v>191</v>
-      </c>
       <c r="L36" s="12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="M36" s="15"/>
       <c r="N36" s="15"/>
@@ -4690,13 +4624,13 @@
         <v>5</v>
       </c>
       <c r="R36" s="12" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="S36" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T36" s="12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="U36" s="12">
         <v>27</v>
@@ -4704,38 +4638,38 @@
     </row>
     <row r="37" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C37" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C37" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D37" s="12">
         <v>56</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F37" s="12" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G37" s="15"/>
       <c r="H37" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="I37" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="J37" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="K37" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="I37" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="J37" s="13" t="s">
-        <v>190</v>
-      </c>
-      <c r="K37" s="13" t="s">
-        <v>191</v>
-      </c>
       <c r="L37" s="12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="M37" s="15"/>
       <c r="N37" s="15"/>
@@ -4745,13 +4679,13 @@
         <v>7</v>
       </c>
       <c r="R37" s="12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="S37" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T37" s="12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="U37" s="12">
         <v>42</v>
@@ -4759,38 +4693,38 @@
     </row>
     <row r="38" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C38" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B38" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C38" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D38" s="12">
         <v>57</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F38" s="12" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G38" s="15"/>
       <c r="H38" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="I38" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="J38" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="K38" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="I38" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="J38" s="13" t="s">
-        <v>190</v>
-      </c>
-      <c r="K38" s="13" t="s">
-        <v>191</v>
-      </c>
       <c r="L38" s="12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="M38" s="15"/>
       <c r="N38" s="15"/>
@@ -4800,13 +4734,13 @@
         <v>8</v>
       </c>
       <c r="R38" s="12" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="S38" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T38" s="12" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="U38" s="12">
         <v>55</v>
@@ -4824,233 +4758,233 @@
   <sheetData>
     <row r="1" spans="1:25" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="K1" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="M1" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="N1" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="R1" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="S1" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="T1" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="U1" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="T1" s="7" t="s">
+      <c r="V1" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="W1" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="V1" s="4" t="s">
+      <c r="X1" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="W1" s="4" t="s">
+      <c r="Y1" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="X1" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y1" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:25" ht="96" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="D2" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="E2" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="F2" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="G2" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="H2" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="I2" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="J2" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="K2" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="L2" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="M2" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="L2" s="9" t="s">
+      <c r="N2" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="O2" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="P2" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="Q2" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="P2" s="8" t="s">
+      <c r="R2" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="Q2" s="8" t="s">
+      <c r="S2" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="R2" s="10" t="s">
+      <c r="T2" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="S2" s="8" t="s">
+      <c r="U2" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="T2" s="10" t="s">
+      <c r="V2" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="U2" s="8" t="s">
+      <c r="W2" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="V2" s="8" t="s">
+      <c r="X2" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="W2" s="8" t="s">
+      <c r="Y2" s="8" t="s">
         <v>76</v>
-      </c>
-      <c r="X2" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="Y2" s="8" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:25" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="P3" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="Q3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="R3" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="S3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="T3" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="U3" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="V3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="W3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="X3" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="Y3" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.2">
@@ -5132,46 +5066,46 @@
     </row>
     <row r="5" spans="1:25" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D5" s="12">
         <v>1</v>
       </c>
       <c r="E5" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="G5" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="H5" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="G5" s="12" t="s">
+      <c r="I5" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="J5" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="I5" s="12" t="s">
+      <c r="K5" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="J5" s="13" t="s">
+      <c r="L5" s="13" t="s">
         <v>89</v>
-      </c>
-      <c r="K5" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="L5" s="13" t="s">
-        <v>91</v>
       </c>
       <c r="M5" s="12">
         <v>39</v>
       </c>
       <c r="N5" s="12" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="O5" s="12">
         <v>35</v>
@@ -5180,24 +5114,24 @@
         <v>46</v>
       </c>
       <c r="Q5" s="12" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="R5" s="12"/>
       <c r="S5" s="12" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="T5" s="14"/>
       <c r="U5" s="12">
         <v>1</v>
       </c>
       <c r="V5" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="W5" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="X5" s="12" t="s">
         <v>95</v>
-      </c>
-      <c r="W5" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="X5" s="12" t="s">
-        <v>97</v>
       </c>
       <c r="Y5" s="12">
         <v>-7</v>
@@ -5205,44 +5139,44 @@
     </row>
     <row r="6" spans="1:25" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D6" s="12">
         <v>2</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="H6" s="12"/>
       <c r="I6" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="J6" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="K6" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="J6" s="13" t="s">
+      <c r="L6" s="13" t="s">
         <v>101</v>
-      </c>
-      <c r="K6" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="L6" s="13" t="s">
-        <v>103</v>
       </c>
       <c r="M6" s="12">
         <v>93</v>
       </c>
       <c r="N6" s="12" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="O6" s="12">
         <v>35</v>
@@ -5251,24 +5185,24 @@
         <v>115</v>
       </c>
       <c r="Q6" s="12" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="R6" s="12"/>
       <c r="S6" s="12" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="T6" s="14"/>
       <c r="U6" s="12">
         <v>1</v>
       </c>
       <c r="V6" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="W6" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="X6" s="12" t="s">
         <v>95</v>
-      </c>
-      <c r="W6" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="X6" s="12" t="s">
-        <v>97</v>
       </c>
       <c r="Y6" s="12">
         <v>-7</v>
@@ -5276,44 +5210,44 @@
     </row>
     <row r="7" spans="1:25" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="D7" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E7" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="F7" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="D7" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="E7" s="12" t="s">
+      <c r="G7" s="12" t="s">
         <v>84</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>86</v>
       </c>
       <c r="H7" s="12"/>
       <c r="I7" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="J7" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K7" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="J7" s="13" t="s">
+      <c r="L7" s="13" t="s">
         <v>89</v>
-      </c>
-      <c r="K7" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="L7" s="13" t="s">
-        <v>91</v>
       </c>
       <c r="M7" s="12">
         <v>39</v>
       </c>
       <c r="N7" s="12" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="O7" s="12">
         <v>35</v>
@@ -5322,24 +5256,24 @@
         <v>46</v>
       </c>
       <c r="Q7" s="12" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="R7" s="12"/>
       <c r="S7" s="12" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="T7" s="14"/>
       <c r="U7" s="12">
         <v>1</v>
       </c>
       <c r="V7" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="W7" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="X7" s="12" t="s">
         <v>95</v>
-      </c>
-      <c r="W7" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="X7" s="12" t="s">
-        <v>97</v>
       </c>
       <c r="Y7" s="12">
         <v>-7</v>

</xml_diff>